<commit_message>
Updated POL_grids_kan50 model - 2026-10-19 23:48
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1880E96-722D-46FE-A91E-CCD91487E9CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF733B43-DB5E-488F-BB34-72B45C66D905}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4183,7 +4183,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D97F03FC-4D63-4B7F-A584-782CA30F930B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B6DF9D9-E725-470A-8333-4A832DD95EC5}">
   <dimension ref="B9:L240"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -33386,7 +33386,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E5A2B79-01E0-4296-9DF3-38E45F0B7C2F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8BD52E-1785-4EC2-A60A-E2CF34981139}">
   <dimension ref="B9:H240"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated POL_grids_kan50 model - 2026-10-20 00:17
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF733B43-DB5E-488F-BB34-72B45C66D905}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{715FA73B-91A1-4729-B13A-2CEA28932869}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4183,7 +4183,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B6DF9D9-E725-470A-8333-4A832DD95EC5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F0F8A21-F33E-4CCB-B215-A216555CFF51}">
   <dimension ref="B9:L240"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -33386,7 +33386,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8BD52E-1785-4EC2-A60A-E2CF34981139}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AE45D6A-A3F8-46DE-B0DD-0BEA25BB22BD}">
   <dimension ref="B9:H240"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated POL_grids_kan50 model - 2026-10-20 00:49
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{715FA73B-91A1-4729-B13A-2CEA28932869}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AA6C366-C387-4E60-AA3A-E5E49FF77BB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4183,7 +4183,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F0F8A21-F33E-4CCB-B215-A216555CFF51}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8461116A-2059-49CB-9DFF-B13EFCFCA5C2}">
   <dimension ref="B9:L240"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -33386,7 +33386,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AE45D6A-A3F8-46DE-B0DD-0BEA25BB22BD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98319A54-4972-4515-A851-960777888CE7}">
   <dimension ref="B9:H240"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated POL_grids_kan50 model - 2026-10-20 10:32
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AA6C366-C387-4E60-AA3A-E5E49FF77BB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7A0B032-A262-40DA-82FB-C53701AA6ED4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4183,7 +4183,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8461116A-2059-49CB-9DFF-B13EFCFCA5C2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E25E6679-EC11-4DD9-8738-91BC6A0D0F1E}">
   <dimension ref="B9:L240"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -33386,7 +33386,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98319A54-4972-4515-A851-960777888CE7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B16D9B5-CD79-4009-B696-29B20F6E7717}">
   <dimension ref="B9:H240"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated POL_grids_kan50 model - 2026-10-20 12:07
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7A0B032-A262-40DA-82FB-C53701AA6ED4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0439DAA-5085-499E-AAE2-BA8FAFCA2E6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4183,7 +4183,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E25E6679-EC11-4DD9-8738-91BC6A0D0F1E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896CC18-0A88-4C55-B273-49C4DBC19257}">
   <dimension ref="B9:L240"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -33386,7 +33386,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B16D9B5-CD79-4009-B696-29B20F6E7717}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7B40D62-A8B4-4307-9706-081AC396E26B}">
   <dimension ref="B9:H240"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated POL_grids_kan50 model - 2026-10-20 20:20
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0439DAA-5085-499E-AAE2-BA8FAFCA2E6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1E9B1CF-80D2-4D36-94AC-F488E603A4A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4183,7 +4183,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896CC18-0A88-4C55-B273-49C4DBC19257}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FA0798F-0635-490A-9C11-FB3E4F5823D1}">
   <dimension ref="B9:L240"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -33386,7 +33386,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7B40D62-A8B4-4307-9706-081AC396E26B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1173826C-9580-4840-BAB9-FCDBC85B31B1}">
   <dimension ref="B9:H240"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated POL_grids_kan50 model - 2026-10-20 21:48
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1E9B1CF-80D2-4D36-94AC-F488E603A4A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98956415-4FC6-446A-80AA-21DD94CC9320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4183,7 +4183,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FA0798F-0635-490A-9C11-FB3E4F5823D1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A296E38-33B5-4BD7-A23E-ED3A787254B9}">
   <dimension ref="B9:L240"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -33386,7 +33386,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1173826C-9580-4840-BAB9-FCDBC85B31B1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7369342C-873D-498F-B7CA-36D0ECFAF487}">
   <dimension ref="B9:H240"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>